<commit_message>
Dapine v2.6 - Fixed DuckDB variables + API auto-flatten + bulletproof filters
</commit_message>
<xml_diff>
--- a/ml_predictions.xlsx
+++ b/ml_predictions.xlsx
@@ -478,7 +478,7 @@
         <v>300000</v>
       </c>
       <c r="E2" t="n">
-        <v>300000</v>
+        <v>307100</v>
       </c>
     </row>
     <row r="3">
@@ -495,7 +495,7 @@
         <v>450000</v>
       </c>
       <c r="E3" t="n">
-        <v>500000</v>
+        <v>447000</v>
       </c>
     </row>
     <row r="4">
@@ -512,7 +512,7 @@
         <v>200000</v>
       </c>
       <c r="E4" t="n">
-        <v>200000</v>
+        <v>229300</v>
       </c>
     </row>
     <row r="5">
@@ -529,7 +529,7 @@
         <v>600000</v>
       </c>
       <c r="E5" t="n">
-        <v>600000</v>
+        <v>581500</v>
       </c>
     </row>
     <row r="6">
@@ -546,7 +546,7 @@
         <v>350000</v>
       </c>
       <c r="E6" t="n">
-        <v>350000</v>
+        <v>343700</v>
       </c>
     </row>
     <row r="7">
@@ -563,7 +563,7 @@
         <v>500000</v>
       </c>
       <c r="E7" t="n">
-        <v>500000</v>
+        <v>487000</v>
       </c>
     </row>
     <row r="8">
@@ -580,7 +580,7 @@
         <v>280000</v>
       </c>
       <c r="E8" t="n">
-        <v>280000</v>
+        <v>271900</v>
       </c>
     </row>
     <row r="9">
@@ -597,7 +597,7 @@
         <v>550000</v>
       </c>
       <c r="E9" t="n">
-        <v>550000</v>
+        <v>546500</v>
       </c>
     </row>
     <row r="10">
@@ -614,7 +614,7 @@
         <v>220000</v>
       </c>
       <c r="E10" t="n">
-        <v>200000</v>
+        <v>249600</v>
       </c>
     </row>
     <row r="11">
@@ -631,7 +631,7 @@
         <v>400000</v>
       </c>
       <c r="E11" t="n">
-        <v>400000</v>
+        <v>386800</v>
       </c>
     </row>
   </sheetData>

</xml_diff>